<commit_message>
22° Commit- aggiornamenti associati al documento per le installazioni manuali  in ambito Patch, aggiornamenti capitoli messaggi/menù locali, aggiornamenti Viste,tabelle diverse, finestre , ws e sottoprogrammi.
</commit_message>
<xml_diff>
--- a/localmenu_message/localMenu-mexsList_protocolCore.xlsx
+++ b/localmenu_message/localMenu-mexsList_protocolCore.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcorbara\Documents\ArgoX3_API_Mobile_CORE\localmenu_message\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A0EB1F-775C-4F3C-BCEE-0B56C798BAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE1E4303-038A-4752-939E-815A2CE3BD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Menù locali- Messaggi" sheetId="1" r:id="rId1"/>
@@ -89,7 +89,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,14 +105,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -260,11 +273,7 @@
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -302,6 +311,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -595,41 +608,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="K2" s="1" t="s">
+      <c r="F2" s="2"/>
+      <c r="K2" s="14" t="s">
         <v>8</v>
       </c>
     </row>
@@ -655,73 +668,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="13">
+      <c r="A3" s="11">
         <v>6203</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="9">
         <v>1</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="9">
         <v>0</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
+      <c r="A4" s="12">
         <v>6203</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="12">
         <v>6203</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
         <v>3</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>2</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15">
+      <c r="A6" s="13">
         <v>6203</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="7">
         <v>4</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="7">
         <v>3</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="8" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>